<commit_message>
feat: add 100-epoch 512x512 experiment 6 and threshold benchmarks
</commit_message>
<xml_diff>
--- a/output metrics.xlsx
+++ b/output metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shrey\Downloads\BTP\CMCNet-main-btp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{188FEE25-E020-4E84-896E-F333B0165424}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{C28FF62E-74DD-49A2-9925-6EB08EC781AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{49DD9F9E-34EF-46C0-A95E-9C85B43366E4}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="21">
   <si>
     <t>Configuration</t>
   </si>
@@ -80,6 +80,15 @@
   </si>
   <si>
     <t>experiment 4</t>
+  </si>
+  <si>
+    <t>experiment 5</t>
+  </si>
+  <si>
+    <t>Original BCE + Dice error (bidirectional gating)</t>
+  </si>
+  <si>
+    <t>threshold: 0.50</t>
   </si>
 </sst>
 </file>
@@ -464,7 +473,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35BF9CAF-0262-4AE5-ACF0-6412061FE120}">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.28515625" bestFit="1" customWidth="1"/>
@@ -472,9 +481,10 @@
     <col min="3" max="3" width="7.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="8" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="8" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="8" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="B1" s="9" t="s">
         <v>0</v>
       </c>
@@ -497,7 +507,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
         <v>6</v>
       </c>
@@ -511,7 +521,7 @@
         <v>13</v>
       </c>
       <c r="E2" s="2">
-        <v>0.92989999999999995</v>
+        <v>0.93</v>
       </c>
       <c r="F2" s="4">
         <v>0.77429999999999999</v>
@@ -523,7 +533,7 @@
         <v>0.8569</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>7</v>
       </c>
@@ -537,7 +547,7 @@
         <v>13</v>
       </c>
       <c r="E3" s="4">
-        <v>0.83309999999999995</v>
+        <v>0.83299999999999996</v>
       </c>
       <c r="F3" s="4">
         <v>0.80479999999999996</v>
@@ -549,7 +559,7 @@
         <v>0.83520000000000005</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -563,7 +573,7 @@
         <v>13</v>
       </c>
       <c r="E4" s="4">
-        <v>0.89739999999999998</v>
+        <v>0.89700000000000002</v>
       </c>
       <c r="F4" s="4">
         <v>0.79600000000000004</v>
@@ -575,7 +585,7 @@
         <v>0.85550000000000004</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -601,29 +611,58 @@
         <v>0.8579</v>
       </c>
     </row>
-    <row r="6" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
+    <row r="6" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="5">
+        <v>20</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6">
+        <v>0.90300000000000002</v>
+      </c>
+      <c r="F6">
+        <v>0.82210000000000005</v>
+      </c>
+      <c r="G6">
+        <v>0.8609</v>
+      </c>
+      <c r="H6">
+        <v>0.86899999999999999</v>
+      </c>
+      <c r="I6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B7" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C7" s="3">
         <v>100</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D7" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E7" s="2">
         <v>0.91200000000000003</v>
       </c>
-      <c r="F6" s="2">
+      <c r="F7" s="2">
         <v>0.8226</v>
       </c>
-      <c r="G6" s="2">
+      <c r="G7" s="2">
         <v>0.86499999999999999</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H7" s="2">
         <v>0.87360000000000004</v>
       </c>
     </row>

</xml_diff>